<commit_message>
[none] Finalize docs/ directory
</commit_message>
<xml_diff>
--- a/docs/20260303-US-group6-emppulse.xlsx
+++ b/docs/20260303-US-group6-emppulse.xlsx
@@ -13,21 +13,21 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={0465a21d-03d4-4abc-9863-e7bad2f9503d}</author>
-    <author>tc={a3568413-88e9-4fd0-817b-9525d5ac3ee9}</author>
-    <author>tc={c64c65ec-cdd0-4507-b36c-a59ce3917926}</author>
+    <author>tc={05988670-3560-43fa-8d2a-5d8038c93ace}</author>
+    <author>tc={94d2dd58-20dd-4077-8695-ab296cd5b007}</author>
+    <author>tc={cbf995a4-1846-4139-8c98-42a34c3078f4}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{0465a21d-03d4-4abc-9863-e7bad2f9503d}" ref="H57">
+    <comment authorId="0" xr:uid="{05988670-3560-43fa-8d2a-5d8038c93ace}" ref="H152">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	combine logic above and current logic in 1
+	At midnight, the system logs a full working day for the following day based on default hours.
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{a3568413-88e9-4fd0-817b-9525d5ac3ee9}" ref="H136">
+    <comment authorId="1" xr:uid="{94d2dd58-20dd-4077-8695-ab296cd5b007}" ref="H136">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -36,12 +36,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{c64c65ec-cdd0-4507-b36c-a59ce3917926}" ref="H152">
+    <comment authorId="2" xr:uid="{cbf995a4-1846-4139-8c98-42a34c3078f4}" ref="H57">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	At midnight, the system logs a full working day for the following day based on default hours.
+	combine logic above and current logic in 1
 </t>
       </text>
     </comment>
@@ -1013,7 +1013,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Andrey Didenko" id="{7e469f0d-3e90-46dd-8e1c-567d503dc0ac}" providerId="google-sheets"/>
+  <x18tc:person displayName="Andrey Didenko" id="{e33a2ea1-a074-4ab0-b232-b8ce079c9363}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1213,13 +1213,13 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="H136" dT="2026-04-23T19:19:42.00" personId="{7e469f0d-3e90-46dd-8e1c-567d503dc0ac}" id="{a3568413-88e9-4fd0-817b-9525d5ac3ee9}" done="1">
+  <x18tc:threadedComment ref="H136" dT="2026-04-23T19:19:42.00" personId="{e33a2ea1-a074-4ab0-b232-b8ce079c9363}" id="{94d2dd58-20dd-4077-8695-ab296cd5b007}" done="1">
     <x18tc:text xml:space="preserve">add working hours</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="H57" dT="2026-04-28T12:40:11.00" personId="{7e469f0d-3e90-46dd-8e1c-567d503dc0ac}" id="{0465a21d-03d4-4abc-9863-e7bad2f9503d}" done="1">
+  <x18tc:threadedComment ref="H57" dT="2026-04-28T12:40:11.00" personId="{e33a2ea1-a074-4ab0-b232-b8ce079c9363}" id="{cbf995a4-1846-4139-8c98-42a34c3078f4}" done="1">
     <x18tc:text xml:space="preserve">combine logic above and current logic in 1</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="H152" dT="2026-04-14T18:09:35.00" personId="{7e469f0d-3e90-46dd-8e1c-567d503dc0ac}" id="{c64c65ec-cdd0-4507-b36c-a59ce3917926}" done="1">
+  <x18tc:threadedComment ref="H152" dT="2026-04-14T18:09:35.00" personId="{e33a2ea1-a074-4ab0-b232-b8ce079c9363}" id="{05988670-3560-43fa-8d2a-5d8038c93ace}" done="1">
     <x18tc:text xml:space="preserve">At midnight, the system logs a full working day for the following day based on default hours.</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -3386,18 +3386,6 @@
     <mergeCell ref="D45:D61"/>
     <mergeCell ref="E45:E61"/>
     <mergeCell ref="F45:F61"/>
-    <mergeCell ref="B86:B92"/>
-    <mergeCell ref="C86:C92"/>
-    <mergeCell ref="D86:D92"/>
-    <mergeCell ref="E86:E92"/>
-    <mergeCell ref="A93:A95"/>
-    <mergeCell ref="B93:B95"/>
-    <mergeCell ref="C93:C95"/>
-    <mergeCell ref="D93:D95"/>
-    <mergeCell ref="E93:E95"/>
-    <mergeCell ref="F93:F95"/>
-    <mergeCell ref="A86:A92"/>
-    <mergeCell ref="F86:F92"/>
     <mergeCell ref="D8:D12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="A2:A7"/>
@@ -3422,6 +3410,8 @@
     <mergeCell ref="D20:D26"/>
     <mergeCell ref="E20:E26"/>
     <mergeCell ref="F20:F26"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
     <mergeCell ref="A27:A31"/>
     <mergeCell ref="B27:B31"/>
     <mergeCell ref="C27:C31"/>
@@ -3433,8 +3423,6 @@
     <mergeCell ref="B141:B144"/>
     <mergeCell ref="C141:C144"/>
     <mergeCell ref="F141:F144"/>
-    <mergeCell ref="D32:D35"/>
-    <mergeCell ref="E32:E35"/>
     <mergeCell ref="D68:D75"/>
     <mergeCell ref="E68:E75"/>
     <mergeCell ref="A62:A67"/>
@@ -3453,8 +3441,20 @@
     <mergeCell ref="E76:E85"/>
     <mergeCell ref="F76:F85"/>
     <mergeCell ref="A76:A85"/>
+    <mergeCell ref="A86:A92"/>
+    <mergeCell ref="B86:B92"/>
+    <mergeCell ref="C86:C92"/>
+    <mergeCell ref="D86:D92"/>
+    <mergeCell ref="E86:E92"/>
+    <mergeCell ref="F86:F92"/>
     <mergeCell ref="D96:D102"/>
     <mergeCell ref="E96:E102"/>
+    <mergeCell ref="A93:A95"/>
+    <mergeCell ref="B93:B95"/>
+    <mergeCell ref="C93:C95"/>
+    <mergeCell ref="D93:D95"/>
+    <mergeCell ref="E93:E95"/>
+    <mergeCell ref="F93:F95"/>
     <mergeCell ref="A96:A102"/>
     <mergeCell ref="F96:F102"/>
     <mergeCell ref="B96:B102"/>

</xml_diff>